<commit_message>
Valor ganado (EVM), portal del cliente, nuevo proyecto y costo unitario en la importación
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Plantilla-importar-actividades.xlsx
+++ b/docs/Plantilla-importar-actividades.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
   <si>
     <t>Frente</t>
   </si>
@@ -45,6 +45,9 @@
     <t>Subcampo</t>
   </si>
   <si>
+    <t>Costo unitario</t>
+  </si>
+  <si>
     <t>BA</t>
   </si>
   <si>
@@ -150,7 +153,10 @@
     <t xml:space="preserve">  Opcionales: Inicio, Fin (fechas dd/mm/aaaa o celdas de fecha), Predecesoras (códigos separados por coma),</t>
   </si>
   <si>
-    <t xml:space="preserve">              Grupo (para el KPI semanal) y Subcampo / Tramo / Sector / Piso (para la matriz por zona).</t>
+    <t xml:space="preserve">              Grupo (para el KPI semanal), Subcampo / Tramo / Sector / Piso (para la matriz por zona)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">              y Costo unitario (costo directo presupuestado por unidad: con él se calcula el valor ganado).</t>
   </si>
   <si>
     <t xml:space="preserve">  El Código no se repite: es lo que une el archivo con la obra cuando vuelvas a importar.</t>
@@ -175,8 +181,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -220,14 +227,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -568,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -579,52 +588,56 @@
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="16" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="1">
         <v>25</v>
@@ -636,27 +649,30 @@
         <v>46340</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="K2" s="3">
+        <v>1800000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="1">
         <v>4200</v>
@@ -668,27 +684,30 @@
         <v>46375</v>
       </c>
       <c r="H3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="3">
+        <v>62000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="1">
         <v>140</v>
@@ -700,27 +719,30 @@
         <v>46403</v>
       </c>
       <c r="H4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" t="s">
         <v>17</v>
       </c>
-      <c r="I4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4" s="3">
+        <v>1450000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1">
         <v>52000</v>
@@ -732,27 +754,30 @@
         <v>46424</v>
       </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="K5" s="3">
+        <v>9500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E6" s="1">
         <v>3800</v>
@@ -764,27 +789,30 @@
         <v>46368</v>
       </c>
       <c r="H6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="3">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
         <v>33</v>
-      </c>
-      <c r="J6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" t="s">
-        <v>32</v>
       </c>
       <c r="E7" s="1">
         <v>7600</v>
@@ -796,13 +824,16 @@
         <v>46410</v>
       </c>
       <c r="H7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J7" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="K7" s="3">
+        <v>7200</v>
       </c>
     </row>
   </sheetData>
@@ -821,23 +852,23 @@
     <col min="3" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>38</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C2">
         <v>4</v>
@@ -845,10 +876,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -862,80 +893,85 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>41</v>
+    <row r="1" spans="1:1" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>